<commit_message>
add fix on prompts llm eval, hotel prompt, add new excel new params hotels_query
</commit_message>
<xml_diff>
--- a/evals/1_inputs/excel/test_dataset_50.xlsx
+++ b/evals/1_inputs/excel/test_dataset_50.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Samuel\Projects\Skripsi\TravelPlanner\TravelPlannerLLMRAGMCP\evals\1_inputs\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicholasterrencesalim/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6CF46F-7B16-4713-A2A8-6BFE1601ADF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{254DB433-7F0D-B548-B16E-D2902F185A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{303DDD28-EEF9-48CD-845F-90282090C77A}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="13900" xr2:uid="{303DDD28-EEF9-48CD-845F-90282090C77A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="148">
   <si>
     <t>id</t>
   </si>
@@ -453,6 +453,36 @@
   </si>
   <si>
     <t>Samosir</t>
+  </si>
+  <si>
+    <t>params_hotels_query</t>
+  </si>
+  <si>
+    <t>Hotel di Bali</t>
+  </si>
+  <si>
+    <t>villa di labuan bajo dekat pusat kota</t>
+  </si>
+  <si>
+    <t>eco resort di likupang</t>
+  </si>
+  <si>
+    <t>hotel bintang 4 di sekitar sirkuit mandalika</t>
+  </si>
+  <si>
+    <t>hotel di Balige yang dekat dengan danau toba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">penginapan murah di bawah 500 ribu per malam dekat Candi Pawon Borobudur </t>
+  </si>
+  <si>
+    <t>hotel keluarga dengan akses langsung ke dermaga kapal di Labuan Bajo</t>
+  </si>
+  <si>
+    <t>Homestay dengan view langsung ke danau toba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resort Bintang 5 di pinggir pantai mandalika lombok </t>
   </si>
 </sst>
 </file>
@@ -820,13 +850,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5431E643-DBFF-44FC-8B03-7A5324952BE6}">
-  <dimension ref="A1:H51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="10" width="13.5546875" customWidth="1"/>
+    <col min="1" max="10" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -851,8 +881,11 @@
       <c r="H1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -863,7 +896,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -874,7 +907,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -885,7 +918,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -896,7 +929,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -907,7 +940,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -918,7 +951,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -929,7 +962,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -940,7 +973,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -951,7 +984,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -962,7 +995,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -973,7 +1006,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -984,7 +1017,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -995,7 +1028,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -1006,7 +1039,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -1017,7 +1050,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -1028,7 +1061,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -1039,7 +1072,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -1050,7 +1083,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -1061,7 +1094,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1072,7 +1105,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1086,7 +1119,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1100,7 +1133,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -1114,7 +1147,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -1128,7 +1161,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>45</v>
       </c>
@@ -1142,7 +1175,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -1156,7 +1189,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>47</v>
       </c>
@@ -1170,7 +1203,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -1184,7 +1217,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -1198,7 +1231,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>50</v>
       </c>
@@ -1212,7 +1245,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>22</v>
       </c>
@@ -1235,7 +1268,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>51</v>
       </c>
@@ -1258,7 +1291,7 @@
         <v>46313</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>52</v>
       </c>
@@ -1281,7 +1314,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>53</v>
       </c>
@@ -1304,7 +1337,7 @@
         <v>46210</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>54</v>
       </c>
@@ -1327,7 +1360,7 @@
         <v>46256</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>55</v>
       </c>
@@ -1347,7 +1380,7 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>56</v>
       </c>
@@ -1367,7 +1400,7 @@
         <v>46283</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>57</v>
       </c>
@@ -1387,7 +1420,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>58</v>
       </c>
@@ -1407,7 +1440,7 @@
         <v>46381</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>59</v>
       </c>
@@ -1427,7 +1460,7 @@
         <v>46208</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>23</v>
       </c>
@@ -1446,8 +1479,11 @@
       <c r="H42" s="1">
         <v>46280</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I42" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>60</v>
       </c>
@@ -1466,8 +1502,11 @@
       <c r="H43" s="1">
         <v>46290</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I43" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>61</v>
       </c>
@@ -1486,8 +1525,11 @@
       <c r="H44" s="1">
         <v>46310</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I44" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>62</v>
       </c>
@@ -1506,8 +1548,11 @@
       <c r="H45" s="1">
         <v>46272</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I45" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>63</v>
       </c>
@@ -1526,8 +1571,11 @@
       <c r="H46" s="1">
         <v>46300</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I46" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>64</v>
       </c>
@@ -1546,8 +1594,11 @@
       <c r="H47" s="1">
         <v>46254</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I47" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>65</v>
       </c>
@@ -1563,8 +1614,11 @@
       <c r="G48" s="1">
         <v>46306</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I48" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>66</v>
       </c>
@@ -1583,8 +1637,11 @@
       <c r="H49" s="1">
         <v>46343</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I49" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>67</v>
       </c>
@@ -1600,8 +1657,11 @@
       <c r="G50" s="1">
         <v>46225</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I50" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>68</v>
       </c>
@@ -1619,6 +1679,9 @@
       </c>
       <c r="H51" s="1">
         <v>46384</v>
+      </c>
+      <c r="I51" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix params in hotels
</commit_message>
<xml_diff>
--- a/evals/1_inputs/excel/test_dataset_50.xlsx
+++ b/evals/1_inputs/excel/test_dataset_50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicholasterrencesalim/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{254DB433-7F0D-B548-B16E-D2902F185A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637BFAB4-6E2C-FE4F-B392-A01C766FA579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="13900" xr2:uid="{303DDD28-EEF9-48CD-845F-90282090C77A}"/>
   </bookViews>
@@ -455,9 +455,6 @@
     <t>Samosir</t>
   </si>
   <si>
-    <t>params_hotels_query</t>
-  </si>
-  <si>
     <t>Hotel di Bali</t>
   </si>
   <si>
@@ -483,6 +480,9 @@
   </si>
   <si>
     <t xml:space="preserve">Resort Bintang 5 di pinggir pantai mandalika lombok </t>
+  </si>
+  <si>
+    <t>param_hotels_query</t>
   </si>
 </sst>
 </file>
@@ -882,7 +882,7 @@
         <v>19</v>
       </c>
       <c r="I1" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -1480,7 +1480,7 @@
         <v>46280</v>
       </c>
       <c r="I42" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
@@ -1503,7 +1503,7 @@
         <v>46290</v>
       </c>
       <c r="I43" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
@@ -1526,7 +1526,7 @@
         <v>46310</v>
       </c>
       <c r="I44" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
@@ -1549,7 +1549,7 @@
         <v>46272</v>
       </c>
       <c r="I45" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
@@ -1572,7 +1572,7 @@
         <v>46300</v>
       </c>
       <c r="I46" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
@@ -1595,7 +1595,7 @@
         <v>46254</v>
       </c>
       <c r="I47" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
@@ -1615,7 +1615,7 @@
         <v>46306</v>
       </c>
       <c r="I48" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
@@ -1638,7 +1638,7 @@
         <v>46343</v>
       </c>
       <c r="I49" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
@@ -1658,7 +1658,7 @@
         <v>46225</v>
       </c>
       <c r="I50" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
@@ -1681,7 +1681,7 @@
         <v>46384</v>
       </c>
       <c r="I51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upadate date on dataset
</commit_message>
<xml_diff>
--- a/evals/1_inputs/excel/test_dataset_50.xlsx
+++ b/evals/1_inputs/excel/test_dataset_50.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicholasterrencesalim/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laura\OneDrive\Attachments\Documents\GitHub\TravelPlannerLLMRAGMCP\evals\1_inputs\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637BFAB4-6E2C-FE4F-B392-A01C766FA579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF9C300F-8EA3-480E-B003-1E75DE1FC3FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="13900" xr2:uid="{303DDD28-EEF9-48CD-845F-90282090C77A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{303DDD28-EEF9-48CD-845F-90282090C77A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -338,54 +338,24 @@
     <t>LOP</t>
   </si>
   <si>
-    <t>Tolong carikan tiket pesawat murah rute Surabaya ke Lombok keberangkatan tanggal 20/09/2026 balik 25/09/2026</t>
-  </si>
-  <si>
     <t>SUB</t>
   </si>
   <si>
-    <t>Cek jadwal pesawat dari Jakarta ke Manado untuk liburan ke Likupang tanggal 15/08/2026 pulang 22/08/2026</t>
-  </si>
-  <si>
     <t>MDC</t>
   </si>
   <si>
     <t>YIA</t>
   </si>
   <si>
-    <t>Ada tidak penerbangan langsung pagi hari dari Makassar ke Lombok untuk tanggal 18/09/2026</t>
-  </si>
-  <si>
     <t>UPG</t>
   </si>
   <si>
     <t>BPN</t>
   </si>
   <si>
-    <t>Cari tiket pesawat transit termurah rute Yogyakarta ke Labuan Bajo tanggal 01/10/2026</t>
-  </si>
-  <si>
-    <t>Cari tiket ke pesawat ke Bali dari Jakarta untuk tanggal 10/09/2026, pulang tanggal 15/09/2026</t>
-  </si>
-  <si>
-    <t>Cari penerbangan kelas bisnis terdekat dari Medan ke Labuan Bajo 05/07/2026</t>
-  </si>
-  <si>
-    <t>Cari tiket sekali jalan dari Balikpapan ke Silangit dengan waktu transit paling singkat tanggal 04/07/2026</t>
-  </si>
-  <si>
     <t>Cek harga tiket pesawat rute Jakarta ke Yogyakarta untuk tanggal 25/12/2026</t>
   </si>
   <si>
-    <t>Cari penerbangan pulang pergi Surabaya ke Manado untuk periode liburan tanggal 27/06/2026 hingga 07/07/2026</t>
-  </si>
-  <si>
-    <t>Cari hotel di Bali untuk tanggal 10/09/2026 sampai 15/09/2026</t>
-  </si>
-  <si>
-    <t>Rekomendasikan resort bintang 5 di pinggir pantai Mandalika Lombok untuk tanggal 20/09/2026 sampai 25/09/2026</t>
-  </si>
-  <si>
     <t>Lombok</t>
   </si>
   <si>
@@ -395,24 +365,15 @@
     <t>Danau Toba</t>
   </si>
   <si>
-    <t>Cari hotel murah di sekitar Borobudur Magelang yang punya fasilitas kolam renang untuk tanggal</t>
-  </si>
-  <si>
     <t>Borobudur</t>
   </si>
   <si>
-    <t>Cari luxury resort atau villa di Labuan Bajo dekat pusat kota untuk tanggal 01/10/2026 sampai 05/10/2026</t>
-  </si>
-  <si>
     <t>Labuan Bajo</t>
   </si>
   <si>
     <t>Likupang</t>
   </si>
   <si>
-    <t>Cari penginapan ramah lingkungan (eco-resort) di kawasan Likupang Sulawesi Utara untuk tanggal 15/08/2026 20/08/2026</t>
-  </si>
-  <si>
     <t>Rekomendasikan hotel bintang 4 di dekat Sirkuit Mandalika yang masih tersedia kamar untuk tanggal</t>
   </si>
   <si>
@@ -425,9 +386,6 @@
     <t>Balige</t>
   </si>
   <si>
-    <t>Tampilkan penginapan murah di bawah 500 ribu per malam dekat Candi Pawon Borobudur untuk tanggal 22/07/2026</t>
-  </si>
-  <si>
     <t>Candi Pawon Borobudur</t>
   </si>
   <si>
@@ -483,6 +441,48 @@
   </si>
   <si>
     <t>param_hotels_query</t>
+  </si>
+  <si>
+    <t>Tampilkan penginapan murah di bawah 500 ribu per malam dekat Candi Pawon Borobudur untuk tanggal 22/10/2026</t>
+  </si>
+  <si>
+    <t>Cari penginapan ramah lingkungan (eco-resort) di kawasan Likupang Sulawesi Utara untuk tanggal 15/10/2026 sampai 20/10/2026</t>
+  </si>
+  <si>
+    <t>Cari luxury resort atau villa di Labuan Bajo dekat pusat kota untuk tanggal 01/11/2026 sampai 05/11/2026</t>
+  </si>
+  <si>
+    <t>Cari hotel murah di sekitar Borobudur Magelang yang punya fasilitas kolam renang untuk tanggal 05/11/2026 sampai 07/11/2026</t>
+  </si>
+  <si>
+    <t>Rekomendasikan resort bintang 5 di pinggir pantai Mandalika Lombok untuk tanggal 20/10/2026 sampai 25/10/2026</t>
+  </si>
+  <si>
+    <t>Cari hotel di Bali untuk tanggal 10/10/2026 sampai 15/10/2026</t>
+  </si>
+  <si>
+    <t>Cari penerbangan kelas bisnis terdekat dari Medan ke Labuan Bajo 05/11/2026</t>
+  </si>
+  <si>
+    <t>Cari tiket sekali jalan dari Balikpapan ke Silangit dengan waktu transit paling singkat tanggal 04/11/2026</t>
+  </si>
+  <si>
+    <t>Ada tidak penerbangan langsung pagi hari dari Makassar ke Lombok untuk tanggal 18/10/2026</t>
+  </si>
+  <si>
+    <t>Cari tiket pesawat transit termurah rute Yogyakarta ke Labuan Bajo tanggal 01/11/2026</t>
+  </si>
+  <si>
+    <t>Cek jadwal pesawat dari Jakarta ke Manado untuk liburan ke Likupang tanggal 15/10/2026 pulang 22/10/2026</t>
+  </si>
+  <si>
+    <t>Cari penerbangan pulang pergi Surabaya ke Manado untuk periode liburan tanggal 27/10/2026 hingga 07/10/2026</t>
+  </si>
+  <si>
+    <t>Tolong carikan tiket pesawat murah rute Surabaya ke Lombok keberangkatan tanggal 20/10/2026 balik 25/10/2026</t>
+  </si>
+  <si>
+    <t>Cari tiket ke pesawat ke Bali dari Jakarta untuk tanggal 10/10/2026, pulang tanggal 15/10/2026</t>
   </si>
 </sst>
 </file>
@@ -532,15 +532,237 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="22">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -851,12 +1073,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5431E643-DBFF-44FC-8B03-7A5324952BE6}">
   <dimension ref="A1:I51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="10" width="13.5" customWidth="1"/>
+    <col min="1" max="2" width="13.42578125" customWidth="1"/>
+    <col min="3" max="3" width="117.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="13.42578125" customWidth="1"/>
+    <col min="7" max="8" width="13.42578125" style="3" customWidth="1"/>
+    <col min="9" max="10" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -882,10 +1108,10 @@
         <v>19</v>
       </c>
       <c r="I1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -895,8 +1121,10 @@
       <c r="C2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G2"/>
+      <c r="H2"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -906,8 +1134,10 @@
       <c r="C3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G3"/>
+      <c r="H3"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -917,8 +1147,10 @@
       <c r="C4" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G4"/>
+      <c r="H4"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -928,8 +1160,10 @@
       <c r="C5" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G5"/>
+      <c r="H5"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -939,8 +1173,10 @@
       <c r="C6" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G6"/>
+      <c r="H6"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -950,8 +1186,10 @@
       <c r="C7" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G7"/>
+      <c r="H7"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -961,8 +1199,10 @@
       <c r="C8" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G8"/>
+      <c r="H8"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -972,8 +1212,10 @@
       <c r="C9" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G9"/>
+      <c r="H9"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -983,8 +1225,10 @@
       <c r="C10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G10"/>
+      <c r="H10"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -994,8 +1238,10 @@
       <c r="C11" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G11"/>
+      <c r="H11"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1005,8 +1251,10 @@
       <c r="C12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G12"/>
+      <c r="H12"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1016,8 +1264,10 @@
       <c r="C13" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G13"/>
+      <c r="H13"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -1027,8 +1277,10 @@
       <c r="C14" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G14"/>
+      <c r="H14"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -1038,8 +1290,10 @@
       <c r="C15" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G15"/>
+      <c r="H15"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>36</v>
       </c>
@@ -1049,8 +1303,10 @@
       <c r="C16" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G16"/>
+      <c r="H16"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -1060,8 +1316,10 @@
       <c r="C17" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G17"/>
+      <c r="H17"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -1071,8 +1329,10 @@
       <c r="C18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G18"/>
+      <c r="H18"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -1082,8 +1342,10 @@
       <c r="C19" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G19"/>
+      <c r="H19"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -1093,8 +1355,10 @@
       <c r="C20" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G20"/>
+      <c r="H20"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1104,8 +1368,10 @@
       <c r="C21" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="G21"/>
+      <c r="H21"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -1116,10 +1382,12 @@
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+      <c r="G22"/>
+      <c r="H22"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -1130,10 +1398,12 @@
         <v>87</v>
       </c>
       <c r="F23" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="G23"/>
+      <c r="H23"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -1144,10 +1414,12 @@
         <v>88</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+      <c r="G24"/>
+      <c r="H24"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -1158,10 +1430,12 @@
         <v>89</v>
       </c>
       <c r="F25" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+      <c r="G25"/>
+      <c r="H25"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>45</v>
       </c>
@@ -1172,10 +1446,12 @@
         <v>90</v>
       </c>
       <c r="F26" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+      <c r="G26"/>
+      <c r="H26"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -1183,13 +1459,15 @@
         <v>8</v>
       </c>
       <c r="C27" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="F27" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+      <c r="G27"/>
+      <c r="H27"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>47</v>
       </c>
@@ -1197,13 +1475,15 @@
         <v>8</v>
       </c>
       <c r="C28" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="F28" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+      <c r="G28"/>
+      <c r="H28"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>48</v>
       </c>
@@ -1214,10 +1494,12 @@
         <v>91</v>
       </c>
       <c r="F29" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+      <c r="G29"/>
+      <c r="H29"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -1228,10 +1510,12 @@
         <v>92</v>
       </c>
       <c r="F30" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+      <c r="G30"/>
+      <c r="H30"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>50</v>
       </c>
@@ -1242,18 +1526,20 @@
         <v>93</v>
       </c>
       <c r="F31" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+        <v>108</v>
+      </c>
+      <c r="G31"/>
+      <c r="H31"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>22</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
       </c>
-      <c r="C32" t="s">
-        <v>108</v>
+      <c r="C32" s="3" t="s">
+        <v>147</v>
       </c>
       <c r="D32" t="s">
         <v>13</v>
@@ -1262,13 +1548,13 @@
         <v>14</v>
       </c>
       <c r="G32" s="1">
-        <v>46275</v>
+        <v>46305</v>
       </c>
       <c r="H32" s="1">
-        <v>46280</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>51</v>
       </c>
@@ -1291,136 +1577,139 @@
         <v>46313</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>52</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D34" t="s">
         <v>99</v>
-      </c>
-      <c r="D34" t="s">
-        <v>100</v>
       </c>
       <c r="E34" t="s">
         <v>98</v>
       </c>
       <c r="G34" s="1">
-        <v>46285</v>
+        <v>46315</v>
       </c>
       <c r="H34" s="1">
-        <v>46290</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46320</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>53</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
       </c>
-      <c r="C35" t="s">
-        <v>112</v>
+      <c r="C35" s="3" t="s">
+        <v>145</v>
       </c>
       <c r="D35" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" t="s">
         <v>100</v>
       </c>
-      <c r="E35" t="s">
-        <v>102</v>
-      </c>
       <c r="G35" s="1">
-        <v>46200</v>
+        <v>46322</v>
       </c>
       <c r="H35" s="1">
-        <v>46210</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46302</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>54</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
       </c>
-      <c r="C36" t="s">
-        <v>101</v>
+      <c r="C36" s="3" t="s">
+        <v>144</v>
       </c>
       <c r="D36" t="s">
         <v>13</v>
       </c>
       <c r="E36" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G36" s="1">
-        <v>46249</v>
+        <v>46310</v>
       </c>
       <c r="H36" s="1">
-        <v>46256</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>55</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
       </c>
-      <c r="C37" t="s">
-        <v>107</v>
+      <c r="C37" s="3" t="s">
+        <v>143</v>
       </c>
       <c r="D37" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>94</v>
       </c>
       <c r="G37" s="1">
-        <v>46296</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46327</v>
+      </c>
+      <c r="H37"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>56</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
       </c>
-      <c r="C38" t="s">
-        <v>104</v>
+      <c r="C38" s="3" t="s">
+        <v>142</v>
       </c>
       <c r="D38" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E38" t="s">
         <v>98</v>
       </c>
       <c r="G38" s="1">
-        <v>46283</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46313</v>
+      </c>
+      <c r="H38"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>57</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
       </c>
-      <c r="C39" t="s">
-        <v>110</v>
+      <c r="C39" s="3" t="s">
+        <v>141</v>
       </c>
       <c r="D39" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E39" t="s">
         <v>96</v>
       </c>
       <c r="G39" s="1">
-        <v>46207</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46330</v>
+      </c>
+      <c r="H39"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>58</v>
       </c>
@@ -1428,27 +1717,28 @@
         <v>9</v>
       </c>
       <c r="C40" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="D40" t="s">
         <v>13</v>
       </c>
       <c r="E40" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G40" s="1">
         <v>46381</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H40"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>59</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
       </c>
-      <c r="C41" t="s">
-        <v>109</v>
+      <c r="C41" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="D41" t="s">
         <v>95</v>
@@ -1457,56 +1747,57 @@
         <v>94</v>
       </c>
       <c r="G41" s="1">
-        <v>46208</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+        <v>46331</v>
+      </c>
+      <c r="H41"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>23</v>
       </c>
       <c r="B42" t="s">
         <v>10</v>
       </c>
-      <c r="C42" t="s">
-        <v>113</v>
+      <c r="C42" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="F42" t="s">
         <v>12</v>
       </c>
       <c r="G42" s="1">
-        <v>46275</v>
+        <v>46305</v>
       </c>
       <c r="H42" s="1">
-        <v>46280</v>
+        <v>46310</v>
       </c>
       <c r="I42" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>60</v>
       </c>
       <c r="B43" t="s">
         <v>10</v>
       </c>
-      <c r="C43" t="s">
-        <v>114</v>
+      <c r="C43" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="F43" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="G43" s="1">
-        <v>46285</v>
+        <v>46315</v>
       </c>
       <c r="H43" s="1">
-        <v>46290</v>
+        <v>46320</v>
       </c>
       <c r="I43" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>61</v>
       </c>
@@ -1514,10 +1805,10 @@
         <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="F44" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="G44" s="1">
         <v>46307</v>
@@ -1526,79 +1817,79 @@
         <v>46310</v>
       </c>
       <c r="I44" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>62</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
       </c>
-      <c r="C45" t="s">
-        <v>118</v>
+      <c r="C45" s="3" t="s">
+        <v>137</v>
       </c>
       <c r="F45" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="G45" s="1">
-        <v>46270</v>
+        <v>46331</v>
       </c>
       <c r="H45" s="1">
-        <v>46272</v>
+        <v>46333</v>
       </c>
       <c r="I45" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>63</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
       </c>
-      <c r="C46" t="s">
-        <v>120</v>
+      <c r="C46" s="3" t="s">
+        <v>136</v>
       </c>
       <c r="F46" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="G46" s="1">
-        <v>46296</v>
+        <v>46327</v>
       </c>
       <c r="H46" s="1">
-        <v>46300</v>
+        <v>46331</v>
       </c>
       <c r="I46" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>64</v>
       </c>
       <c r="B47" t="s">
         <v>10</v>
       </c>
-      <c r="C47" t="s">
-        <v>123</v>
+      <c r="C47" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="F47" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="G47" s="1">
-        <v>46249</v>
+        <v>46310</v>
       </c>
       <c r="H47" s="1">
-        <v>46254</v>
+        <v>46315</v>
       </c>
       <c r="I47" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>65</v>
       </c>
@@ -1606,19 +1897,20 @@
         <v>10</v>
       </c>
       <c r="C48" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="F48" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="G48" s="1">
         <v>46306</v>
       </c>
+      <c r="H48"/>
       <c r="I48" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>66</v>
       </c>
@@ -1626,10 +1918,10 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="F49" t="s">
-        <v>127</v>
+        <v>114</v>
       </c>
       <c r="G49" s="1">
         <v>46340</v>
@@ -1638,30 +1930,31 @@
         <v>46343</v>
       </c>
       <c r="I49" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>67</v>
       </c>
       <c r="B50" t="s">
         <v>10</v>
       </c>
-      <c r="C50" t="s">
-        <v>128</v>
+      <c r="C50" s="3" t="s">
+        <v>134</v>
       </c>
       <c r="F50" t="s">
+        <v>115</v>
+      </c>
+      <c r="G50" s="1">
+        <v>46317</v>
+      </c>
+      <c r="H50"/>
+      <c r="I50" t="s">
         <v>129</v>
       </c>
-      <c r="G50" s="1">
-        <v>46225</v>
-      </c>
-      <c r="I50" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>68</v>
       </c>
@@ -1669,10 +1962,10 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="F51" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="G51" s="1">
         <v>46380</v>
@@ -1681,7 +1974,7 @@
         <v>46384</v>
       </c>
       <c r="I51" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>